<commit_message>
RHU planillas y DSI U3
</commit_message>
<xml_diff>
--- a/Ciclo 01/RHU/Ejercicio taller.xlsx
+++ b/Ciclo 01/RHU/Ejercicio taller.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vasqu\OneDrive\Escritorio\Recursos Humanos 2026\UNIDAD II\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luizi\OneDrive\Escritorio\UES-2026\Ciclo 01\RHU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6946065-D73C-4371-9D97-52C9317E6367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F87A31DB-9CBF-45CC-A49B-A6B2BE3C27BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planteamiento" sheetId="3" r:id="rId1"/>
@@ -18,11 +18,22 @@
     <sheet name="EjercicioPlanilla-Solución" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="92">
   <si>
     <t>AREA</t>
   </si>
@@ -550,14 +561,56 @@
   <si>
     <t>Monto a depositar planilla única</t>
   </si>
+  <si>
+    <t>Años trabajados</t>
+  </si>
+  <si>
+    <t>Precio Hora</t>
+  </si>
+  <si>
+    <t>Horas Extras Diurnas</t>
+  </si>
+  <si>
+    <t>Horas Extras Nocturnas</t>
+  </si>
+  <si>
+    <t>Vacaciones</t>
+  </si>
+  <si>
+    <t>Bonificacion Vacaciones</t>
+  </si>
+  <si>
+    <t>Aguinaldo</t>
+  </si>
+  <si>
+    <t>Bonificacion Aguinaldo</t>
+  </si>
+  <si>
+    <t>Monto Cotizable</t>
+  </si>
+  <si>
+    <t>ISSS Patronal 7,5%</t>
+  </si>
+  <si>
+    <t>ISSS Empleado 3%</t>
+  </si>
+  <si>
+    <t>Monto Planilla unica</t>
+  </si>
+  <si>
+    <t>AFP Patronal 8,75%</t>
+  </si>
+  <si>
+    <t>AFP Empleado 7,25%</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -636,7 +689,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -667,8 +720,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -775,33 +840,44 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -834,10 +910,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -855,7 +931,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -879,7 +955,7 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -898,28 +974,25 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="2" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -928,16 +1001,16 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="44" fontId="2" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -953,23 +1026,43 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="10" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1294,284 +1387,291 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C3" s="57" t="s">
+      <c r="C3" s="56" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="4" spans="2:5" ht="45" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="62" t="s">
+      <c r="C4" s="58" t="s">
         <v>72</v>
       </c>
-      <c r="D4" s="62"/>
-      <c r="E4" s="62"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C6" s="63" t="s">
+      <c r="C6" s="59" t="s">
         <v>60</v>
       </c>
-      <c r="D6" s="63"/>
-      <c r="E6" s="63"/>
+      <c r="D6" s="59"/>
+      <c r="E6" s="59"/>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B8" s="58">
+      <c r="B8" s="57">
         <v>1</v>
       </c>
-      <c r="C8" s="58" t="s">
+      <c r="C8" s="57" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="58" t="s">
+      <c r="D8" s="57" t="s">
         <v>53</v>
       </c>
-      <c r="E8" s="58" t="s">
+      <c r="E8" s="57" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B9" s="58">
+      <c r="B9" s="57">
         <v>2</v>
       </c>
-      <c r="C9" s="58" t="s">
+      <c r="C9" s="57" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="58" t="s">
+      <c r="D9" s="57" t="s">
         <v>53</v>
       </c>
-      <c r="E9" s="58" t="s">
+      <c r="E9" s="57" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="B10" s="58">
+      <c r="B10" s="57">
         <v>3</v>
       </c>
-      <c r="C10" s="58" t="s">
+      <c r="C10" s="57" t="s">
         <v>59</v>
       </c>
-      <c r="D10" s="58" t="s">
+      <c r="D10" s="57" t="s">
         <v>53</v>
       </c>
-      <c r="E10" s="58" t="s">
+      <c r="E10" s="57" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="C12" s="64" t="s">
+      <c r="C12" s="60" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="64"/>
-      <c r="E12" s="64"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="60"/>
     </row>
     <row r="15" spans="2:5" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C15" s="62" t="s">
+      <c r="C15" s="58" t="s">
         <v>62</v>
       </c>
-      <c r="D15" s="62"/>
-      <c r="E15" s="62"/>
+      <c r="D15" s="58"/>
+      <c r="E15" s="58"/>
     </row>
     <row r="16" spans="2:5" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="61" t="s">
+      <c r="C16" s="66" t="s">
         <v>63</v>
       </c>
-      <c r="D16" s="61"/>
-      <c r="E16" s="61"/>
+      <c r="D16" s="66"/>
+      <c r="E16" s="66"/>
     </row>
     <row r="17" spans="2:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C17" s="61" t="s">
+      <c r="C17" s="66" t="s">
         <v>64</v>
       </c>
-      <c r="D17" s="61"/>
-      <c r="E17" s="61"/>
+      <c r="D17" s="66"/>
+      <c r="E17" s="66"/>
     </row>
     <row r="18" spans="2:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C18" s="61" t="s">
+      <c r="C18" s="66" t="s">
         <v>65</v>
       </c>
-      <c r="D18" s="61"/>
-      <c r="E18" s="61"/>
+      <c r="D18" s="66"/>
+      <c r="E18" s="66"/>
     </row>
     <row r="19" spans="2:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="61" t="s">
+      <c r="C19" s="66" t="s">
         <v>69</v>
       </c>
-      <c r="D19" s="61"/>
-      <c r="E19" s="61"/>
+      <c r="D19" s="66"/>
+      <c r="E19" s="66"/>
     </row>
     <row r="20" spans="2:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C20" s="61" t="s">
+      <c r="C20" s="66" t="s">
         <v>70</v>
       </c>
-      <c r="D20" s="61"/>
-      <c r="E20" s="61"/>
+      <c r="D20" s="66"/>
+      <c r="E20" s="66"/>
     </row>
     <row r="21" spans="2:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="61" t="s">
+      <c r="C21" s="66" t="s">
         <v>66</v>
       </c>
-      <c r="D21" s="61"/>
-      <c r="E21" s="61"/>
+      <c r="D21" s="66"/>
+      <c r="E21" s="66"/>
     </row>
     <row r="22" spans="2:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C22" s="61" t="s">
+      <c r="C22" s="66" t="s">
         <v>73</v>
       </c>
-      <c r="D22" s="61"/>
-      <c r="E22" s="61"/>
+      <c r="D22" s="66"/>
+      <c r="E22" s="66"/>
     </row>
     <row r="23" spans="2:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C23" s="61" t="s">
+      <c r="C23" s="66" t="s">
         <v>74</v>
       </c>
-      <c r="D23" s="61"/>
-      <c r="E23" s="61"/>
+      <c r="D23" s="66"/>
+      <c r="E23" s="66"/>
     </row>
     <row r="24" spans="2:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C24" s="61" t="s">
+      <c r="C24" s="66" t="s">
         <v>67</v>
       </c>
-      <c r="D24" s="61"/>
-      <c r="E24" s="61"/>
+      <c r="D24" s="66"/>
+      <c r="E24" s="66"/>
     </row>
     <row r="25" spans="2:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C25" s="61" t="s">
+      <c r="C25" s="66" t="s">
         <v>75</v>
       </c>
-      <c r="D25" s="61"/>
-      <c r="E25" s="61"/>
+      <c r="D25" s="66"/>
+      <c r="E25" s="66"/>
     </row>
     <row r="26" spans="2:5" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C26" s="61" t="s">
+      <c r="C26" s="66" t="s">
         <v>76</v>
       </c>
-      <c r="D26" s="61"/>
-      <c r="E26" s="61"/>
+      <c r="D26" s="66"/>
+      <c r="E26" s="66"/>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B31" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="C31" s="60" t="s">
+      <c r="C31" s="61" t="s">
         <v>35</v>
       </c>
-      <c r="D31" s="60"/>
-      <c r="E31" s="60"/>
+      <c r="D31" s="61"/>
+      <c r="E31" s="61"/>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B32" s="38">
         <v>1</v>
       </c>
-      <c r="C32" s="59" t="s">
+      <c r="C32" s="69" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="59"/>
-      <c r="E32" s="59"/>
+      <c r="D32" s="69"/>
+      <c r="E32" s="69"/>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B33" s="38">
         <v>2</v>
       </c>
-      <c r="C33" s="59" t="s">
+      <c r="C33" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="D33" s="59"/>
-      <c r="E33" s="59"/>
+      <c r="D33" s="69"/>
+      <c r="E33" s="69"/>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B34" s="38">
         <v>3</v>
       </c>
-      <c r="C34" s="59" t="s">
+      <c r="C34" s="69" t="s">
         <v>42</v>
       </c>
-      <c r="D34" s="59"/>
-      <c r="E34" s="59"/>
+      <c r="D34" s="69"/>
+      <c r="E34" s="69"/>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B35" s="38">
         <v>4</v>
       </c>
-      <c r="C35" s="59" t="s">
+      <c r="C35" s="69" t="s">
         <v>43</v>
       </c>
-      <c r="D35" s="59"/>
-      <c r="E35" s="59"/>
+      <c r="D35" s="69"/>
+      <c r="E35" s="69"/>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B36" s="38">
         <v>5</v>
       </c>
-      <c r="C36" s="59" t="s">
+      <c r="C36" s="69" t="s">
         <v>44</v>
       </c>
-      <c r="D36" s="59"/>
-      <c r="E36" s="59"/>
+      <c r="D36" s="69"/>
+      <c r="E36" s="69"/>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B37" s="38">
         <v>6</v>
       </c>
-      <c r="C37" s="59" t="s">
+      <c r="C37" s="69" t="s">
         <v>37</v>
       </c>
-      <c r="D37" s="59"/>
-      <c r="E37" s="59"/>
+      <c r="D37" s="69"/>
+      <c r="E37" s="69"/>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B38" s="38">
         <v>7</v>
       </c>
-      <c r="C38" s="59" t="s">
+      <c r="C38" s="69" t="s">
         <v>38</v>
       </c>
-      <c r="D38" s="59"/>
-      <c r="E38" s="59"/>
+      <c r="D38" s="69"/>
+      <c r="E38" s="69"/>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B39" s="38">
         <v>8</v>
       </c>
-      <c r="C39" s="59" t="s">
+      <c r="C39" s="69" t="s">
         <v>39</v>
       </c>
-      <c r="D39" s="59"/>
-      <c r="E39" s="59"/>
+      <c r="D39" s="69"/>
+      <c r="E39" s="69"/>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B40" s="38">
         <v>9</v>
       </c>
-      <c r="C40" s="59" t="s">
+      <c r="C40" s="69" t="s">
         <v>40</v>
       </c>
-      <c r="D40" s="59"/>
-      <c r="E40" s="59"/>
+      <c r="D40" s="69"/>
+      <c r="E40" s="69"/>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B41" s="38">
         <v>10</v>
       </c>
-      <c r="C41" s="59" t="s">
+      <c r="C41" s="62" t="s">
         <v>45</v>
       </c>
-      <c r="D41" s="59"/>
-      <c r="E41" s="59"/>
+      <c r="D41" s="62"/>
+      <c r="E41" s="62"/>
     </row>
     <row r="42" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="38">
         <v>11</v>
       </c>
-      <c r="C42" s="59" t="s">
+      <c r="C42" s="62" t="s">
         <v>46</v>
       </c>
-      <c r="D42" s="59"/>
-      <c r="E42" s="59"/>
+      <c r="D42" s="62"/>
+      <c r="E42" s="62"/>
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="C6:E6"/>
-    <mergeCell ref="C12:E12"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="C42:E42"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="C31:E31"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="C35:E35"/>
     <mergeCell ref="C17:E17"/>
     <mergeCell ref="C18:E18"/>
     <mergeCell ref="C19:E19"/>
@@ -1582,18 +1682,11 @@
     <mergeCell ref="C23:E23"/>
     <mergeCell ref="C24:E24"/>
     <mergeCell ref="C25:E25"/>
-    <mergeCell ref="C31:E31"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="C34:E34"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="C41:E41"/>
-    <mergeCell ref="C42:E42"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="C39:E39"/>
-    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C16:E16"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="textLength" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B31:C42" xr:uid="{B2AC17C9-1910-4260-AA3A-E76C21A97FA1}">
@@ -1606,34 +1699,39 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56A14A74-6763-4EAC-B4D1-B2430F5A4CAB}">
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:W18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.6640625" customWidth="1"/>
     <col min="4" max="5" width="12.33203125" customWidth="1"/>
-    <col min="7" max="9" width="13.109375" customWidth="1"/>
-    <col min="11" max="11" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.109375" customWidth="1"/>
+    <col min="8" max="8" width="4.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
+    <col min="12" max="12" width="12.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
       <c r="G1" s="24"/>
       <c r="H1" s="24"/>
       <c r="I1" s="24"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J1" s="24"/>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="G2" s="25"/>
       <c r="H2" s="25"/>
       <c r="I2" s="25"/>
-    </row>
-    <row r="4" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J2" s="25"/>
+    </row>
+    <row r="4" spans="1:23" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B4" s="34" t="s">
         <v>68</v>
       </c>
       <c r="C4" s="34"/>
     </row>
-    <row r="5" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -1655,8 +1753,56 @@
       <c r="G5" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H5" s="63" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5" s="63" t="s">
+        <v>78</v>
+      </c>
+      <c r="J5" s="63" t="s">
+        <v>79</v>
+      </c>
+      <c r="K5" s="70" t="s">
+        <v>80</v>
+      </c>
+      <c r="L5" s="70" t="s">
+        <v>81</v>
+      </c>
+      <c r="M5" s="70" t="s">
+        <v>82</v>
+      </c>
+      <c r="N5" s="70" t="s">
+        <v>83</v>
+      </c>
+      <c r="O5" s="70" t="s">
+        <v>84</v>
+      </c>
+      <c r="P5" s="70" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q5" s="70" t="s">
+        <v>86</v>
+      </c>
+      <c r="R5" s="70" t="s">
+        <v>87</v>
+      </c>
+      <c r="S5" s="70" t="s">
+        <v>88</v>
+      </c>
+      <c r="T5" s="70" t="s">
+        <v>90</v>
+      </c>
+      <c r="U5" s="70" t="s">
+        <v>91</v>
+      </c>
+      <c r="V5" s="70" t="s">
+        <v>33</v>
+      </c>
+      <c r="W5" s="70" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>1</v>
       </c>
@@ -1678,8 +1824,70 @@
       <c r="G6" s="2">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H6" s="64">
+        <f>MONTH(D6)</f>
+        <v>12</v>
+      </c>
+      <c r="I6" s="65">
+        <f>(E6-D6)/365</f>
+        <v>13.09041095890411</v>
+      </c>
+      <c r="J6" s="2">
+        <f>+(F6/30)/8</f>
+        <v>6.666666666666667</v>
+      </c>
+      <c r="K6" s="2">
+        <v>0</v>
+      </c>
+      <c r="L6" s="2">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2">
+        <f>IF(H6=12,(F6/2)*30%,0)</f>
+        <v>240</v>
+      </c>
+      <c r="N6" s="2">
+        <f>IF($H6=12,IF((AND($I6&gt;=2,$I6&lt;5)),(($F6/2)*5%),IF($I6&gt;=5,(($F6/2)*15%),0)),0)</f>
+        <v>120</v>
+      </c>
+      <c r="O6" s="2">
+        <f>IF((AND($I6&gt;=1,$I6&lt;3)),((F6/30)*15),IF((AND($I6&gt;=3,$I6&lt;10)),((F6/30)*19),((F6/30)*21)))</f>
+        <v>1120</v>
+      </c>
+      <c r="P6" s="2">
+        <f>IF(I6&gt;3,F6-O6,0)</f>
+        <v>480</v>
+      </c>
+      <c r="Q6" s="2">
+        <f>+F6+K6+L6+M6+N6</f>
+        <v>1960</v>
+      </c>
+      <c r="R6" s="2">
+        <f>IF(Q6&gt;1000,1000*7.5%,Q6*7.5%)</f>
+        <v>75</v>
+      </c>
+      <c r="S6" s="2">
+        <f>IF(Q6&gt;1000,1000*3%,Q6*3%)</f>
+        <v>30</v>
+      </c>
+      <c r="T6" s="2">
+        <f>+Q6*8.75%</f>
+        <v>171.5</v>
+      </c>
+      <c r="U6" s="2">
+        <f>+Q6*7.25%</f>
+        <v>142.1</v>
+      </c>
+      <c r="V6" s="2">
+        <f>+G6+O6+P6+Q6-S6-U6</f>
+        <v>3412.9</v>
+      </c>
+      <c r="W6" s="2">
+        <f>+R6+S6+T6+U6</f>
+        <v>418.6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <f>+A6+1</f>
         <v>2</v>
@@ -1704,10 +1912,72 @@
         <f>+G6</f>
         <v>25</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H7" s="64">
+        <f t="shared" ref="H7:H16" si="0">MONTH(D7)</f>
+        <v>8</v>
+      </c>
+      <c r="I7" s="65">
+        <f t="shared" ref="I7:I16" si="1">(E7-D7)/365</f>
+        <v>7.3561643835616435</v>
+      </c>
+      <c r="J7" s="2">
+        <f t="shared" ref="J7:J16" si="2">+(F7/30)/8</f>
+        <v>2.0833333333333335</v>
+      </c>
+      <c r="K7" s="2">
+        <v>0</v>
+      </c>
+      <c r="L7" s="2">
+        <v>0</v>
+      </c>
+      <c r="M7" s="2">
+        <f t="shared" ref="M7:M16" si="3">IF(H7=12,(F7/2)*30%,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N7" s="2">
+        <f t="shared" ref="N7:N16" si="4">IF($H7=12,IF((AND($I7&gt;=2,$I7&lt;5)),(($F7/2)*5%),IF($I7&gt;=5,(($F7/2)*15%),0)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="O7" s="2">
+        <f t="shared" ref="O7:O16" si="5">IF((AND($I7&gt;=1,$I7&lt;3)),((F7/30)*15),IF((AND($I7&gt;=3,$I7&lt;10)),((F7/30)*19),((F7/30)*21)))</f>
+        <v>316.66666666666669</v>
+      </c>
+      <c r="P7" s="2">
+        <f t="shared" ref="P7:P16" si="6">IF(I7&gt;3,F7-O7,0)</f>
+        <v>183.33333333333331</v>
+      </c>
+      <c r="Q7" s="2">
+        <f t="shared" ref="Q7:Q16" si="7">+F7+K7+L7+M7+N7</f>
+        <v>500</v>
+      </c>
+      <c r="R7" s="2">
+        <f t="shared" ref="R7:R16" si="8">IF(Q7&gt;1000,1000*7.5%,Q7*7.5%)</f>
+        <v>37.5</v>
+      </c>
+      <c r="S7" s="2">
+        <f t="shared" ref="S7:S16" si="9">IF(Q7&gt;1000,1000*3%,Q7*3%)</f>
+        <v>15</v>
+      </c>
+      <c r="T7" s="2">
+        <f t="shared" ref="T7:T16" si="10">+Q7*8.75%</f>
+        <v>43.75</v>
+      </c>
+      <c r="U7" s="2">
+        <f t="shared" ref="U7:U16" si="11">+Q7*7.25%</f>
+        <v>36.25</v>
+      </c>
+      <c r="V7" s="2">
+        <f t="shared" ref="V7:V16" si="12">+G7+O7+P7+Q7-S7-U7</f>
+        <v>973.75</v>
+      </c>
+      <c r="W7" s="2">
+        <f t="shared" ref="W7:W16" si="13">+R7+S7+T7+U7</f>
+        <v>132.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
-        <f t="shared" ref="A8:A16" si="0">+A7+1</f>
+        <f t="shared" ref="A8:A16" si="14">+A7+1</f>
         <v>3</v>
       </c>
       <c r="B8" s="26" t="s">
@@ -1720,7 +1990,7 @@
         <v>43801</v>
       </c>
       <c r="E8" s="10">
-        <f t="shared" ref="E8:E9" si="1">+E7</f>
+        <f t="shared" ref="E8:E9" si="15">+E7</f>
         <v>46022</v>
       </c>
       <c r="F8" s="2">
@@ -1730,10 +2000,72 @@
         <f>+G7</f>
         <v>25</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" s="13" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H8" s="64">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="I8" s="65">
+        <f t="shared" si="1"/>
+        <v>6.0849315068493155</v>
+      </c>
+      <c r="J8" s="2">
+        <f t="shared" si="2"/>
+        <v>2.8125</v>
+      </c>
+      <c r="K8" s="2">
+        <v>0</v>
+      </c>
+      <c r="L8" s="2">
+        <v>0</v>
+      </c>
+      <c r="M8" s="2">
+        <f t="shared" si="3"/>
+        <v>101.25</v>
+      </c>
+      <c r="N8" s="2">
+        <f t="shared" si="4"/>
+        <v>50.625</v>
+      </c>
+      <c r="O8" s="2">
+        <f t="shared" si="5"/>
+        <v>427.5</v>
+      </c>
+      <c r="P8" s="2">
+        <f t="shared" si="6"/>
+        <v>247.5</v>
+      </c>
+      <c r="Q8" s="2">
+        <f t="shared" si="7"/>
+        <v>826.875</v>
+      </c>
+      <c r="R8" s="2">
+        <f t="shared" si="8"/>
+        <v>62.015625</v>
+      </c>
+      <c r="S8" s="2">
+        <f t="shared" si="9"/>
+        <v>24.806249999999999</v>
+      </c>
+      <c r="T8" s="2">
+        <f t="shared" si="10"/>
+        <v>72.3515625</v>
+      </c>
+      <c r="U8" s="2">
+        <f t="shared" si="11"/>
+        <v>59.948437499999997</v>
+      </c>
+      <c r="V8" s="2">
+        <f t="shared" si="12"/>
+        <v>1442.1203125</v>
+      </c>
+      <c r="W8" s="2">
+        <f t="shared" si="13"/>
+        <v>219.12187499999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" s="13" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="14"/>
         <v>4</v>
       </c>
       <c r="B9" s="27" t="s">
@@ -1746,22 +2078,80 @@
         <v>44146</v>
       </c>
       <c r="E9" s="10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="15"/>
         <v>46022</v>
       </c>
       <c r="F9" s="2">
         <v>750</v>
       </c>
       <c r="G9" s="2">
-        <f t="shared" ref="G9" si="2">+G8</f>
+        <f t="shared" ref="G9" si="16">+G8</f>
         <v>25</v>
       </c>
-      <c r="H9"/>
-      <c r="I9"/>
-      <c r="J9"/>
-      <c r="K9"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H9" s="64">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="I9" s="65">
+        <f t="shared" si="1"/>
+        <v>5.13972602739726</v>
+      </c>
+      <c r="J9" s="2">
+        <f t="shared" si="2"/>
+        <v>3.125</v>
+      </c>
+      <c r="K9" s="2">
+        <v>0</v>
+      </c>
+      <c r="L9" s="2">
+        <v>0</v>
+      </c>
+      <c r="M9" s="2">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N9" s="2">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="O9" s="2">
+        <f t="shared" si="5"/>
+        <v>475</v>
+      </c>
+      <c r="P9" s="2">
+        <f t="shared" si="6"/>
+        <v>275</v>
+      </c>
+      <c r="Q9" s="2">
+        <f t="shared" si="7"/>
+        <v>750</v>
+      </c>
+      <c r="R9" s="2">
+        <f t="shared" si="8"/>
+        <v>56.25</v>
+      </c>
+      <c r="S9" s="2">
+        <f t="shared" si="9"/>
+        <v>22.5</v>
+      </c>
+      <c r="T9" s="2">
+        <f t="shared" si="10"/>
+        <v>65.625</v>
+      </c>
+      <c r="U9" s="2">
+        <f t="shared" si="11"/>
+        <v>54.374999999999993</v>
+      </c>
+      <c r="V9" s="2">
+        <f t="shared" si="12"/>
+        <v>1448.125</v>
+      </c>
+      <c r="W9" s="2">
+        <f t="shared" si="13"/>
+        <v>198.75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
       <c r="B10" s="26"/>
       <c r="C10" s="22"/>
@@ -1777,8 +2167,63 @@
         <f>SUM(G6:G9)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H10" s="64"/>
+      <c r="I10" s="65"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="5">
+        <f>SUM(K6:K9)</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="5">
+        <f>SUM(L6:L9)</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="5">
+        <f>SUM(M6:M9)</f>
+        <v>341.25</v>
+      </c>
+      <c r="N10" s="5">
+        <f>SUM(N6:N9)</f>
+        <v>170.625</v>
+      </c>
+      <c r="O10" s="5">
+        <f>SUM(O6:O9)</f>
+        <v>2339.166666666667</v>
+      </c>
+      <c r="P10" s="5">
+        <f>SUM(P6:P9)</f>
+        <v>1185.8333333333333</v>
+      </c>
+      <c r="Q10" s="5">
+        <f>SUM(Q6:Q9)</f>
+        <v>4036.875</v>
+      </c>
+      <c r="R10" s="5">
+        <f t="shared" ref="R10:S10" si="17">SUM(R6:R9)</f>
+        <v>230.765625</v>
+      </c>
+      <c r="S10" s="5">
+        <f t="shared" si="17"/>
+        <v>92.306250000000006</v>
+      </c>
+      <c r="T10" s="5">
+        <f t="shared" ref="T10" si="18">SUM(T6:T9)</f>
+        <v>353.2265625</v>
+      </c>
+      <c r="U10" s="5">
+        <f t="shared" ref="U10" si="19">SUM(U6:U9)</f>
+        <v>292.67343749999998</v>
+      </c>
+      <c r="V10" s="5">
+        <f t="shared" ref="V10" si="20">SUM(V6:V9)</f>
+        <v>7276.8953124999998</v>
+      </c>
+      <c r="W10" s="5">
+        <f t="shared" ref="W10" si="21">SUM(W6:W9)</f>
+        <v>968.97187499999995</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <f>+A9+1</f>
         <v>5</v>
@@ -1802,10 +2247,72 @@
       <c r="G11" s="2">
         <v>35</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H11" s="64">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="I11" s="65">
+        <f t="shared" si="1"/>
+        <v>8.493150684931507</v>
+      </c>
+      <c r="J11" s="2">
+        <f t="shared" si="2"/>
+        <v>1.9791666666666667</v>
+      </c>
+      <c r="K11" s="2">
+        <v>0</v>
+      </c>
+      <c r="L11" s="2">
+        <v>0</v>
+      </c>
+      <c r="M11" s="2">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N11" s="2">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="O11" s="2">
+        <f t="shared" si="5"/>
+        <v>300.83333333333337</v>
+      </c>
+      <c r="P11" s="2">
+        <f t="shared" si="6"/>
+        <v>174.16666666666663</v>
+      </c>
+      <c r="Q11" s="2">
+        <f t="shared" si="7"/>
+        <v>475</v>
+      </c>
+      <c r="R11" s="2">
+        <f t="shared" si="8"/>
+        <v>35.625</v>
+      </c>
+      <c r="S11" s="2">
+        <f t="shared" si="9"/>
+        <v>14.25</v>
+      </c>
+      <c r="T11" s="2">
+        <f t="shared" si="10"/>
+        <v>41.5625</v>
+      </c>
+      <c r="U11" s="2">
+        <f t="shared" si="11"/>
+        <v>34.4375</v>
+      </c>
+      <c r="V11" s="2">
+        <f t="shared" si="12"/>
+        <v>936.3125</v>
+      </c>
+      <c r="W11" s="2">
+        <f t="shared" si="13"/>
+        <v>125.875</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="14"/>
         <v>6</v>
       </c>
       <c r="B12" s="26" t="s">
@@ -1828,62 +2335,250 @@
         <f>+G11</f>
         <v>35</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H12" s="64">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="I12" s="65">
+        <f t="shared" si="1"/>
+        <v>5.8219178082191778</v>
+      </c>
+      <c r="J12" s="2">
+        <f t="shared" si="2"/>
+        <v>1.7708333333333333</v>
+      </c>
+      <c r="K12" s="2">
+        <v>0</v>
+      </c>
+      <c r="L12" s="2">
+        <v>0</v>
+      </c>
+      <c r="M12" s="2">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N12" s="2">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="O12" s="2">
+        <f t="shared" si="5"/>
+        <v>269.16666666666663</v>
+      </c>
+      <c r="P12" s="2">
+        <f t="shared" si="6"/>
+        <v>155.83333333333337</v>
+      </c>
+      <c r="Q12" s="2">
+        <f t="shared" si="7"/>
+        <v>425</v>
+      </c>
+      <c r="R12" s="2">
+        <f t="shared" si="8"/>
+        <v>31.875</v>
+      </c>
+      <c r="S12" s="2">
+        <f t="shared" si="9"/>
+        <v>12.75</v>
+      </c>
+      <c r="T12" s="2">
+        <f t="shared" si="10"/>
+        <v>37.1875</v>
+      </c>
+      <c r="U12" s="2">
+        <f t="shared" si="11"/>
+        <v>30.812499999999996</v>
+      </c>
+      <c r="V12" s="2">
+        <f t="shared" si="12"/>
+        <v>841.4375</v>
+      </c>
+      <c r="W12" s="2">
+        <f t="shared" si="13"/>
+        <v>112.625</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
+        <f t="shared" si="14"/>
+        <v>7</v>
+      </c>
+      <c r="B13" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="12">
+        <v>43807</v>
+      </c>
+      <c r="E13" s="10">
+        <f t="shared" ref="E13:E16" si="22">+E12</f>
+        <v>46022</v>
+      </c>
+      <c r="F13" s="2">
+        <v>450</v>
+      </c>
+      <c r="G13" s="2">
+        <f t="shared" ref="G13:G16" si="23">+G11</f>
+        <v>35</v>
+      </c>
+      <c r="H13" s="64">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="I13" s="65">
+        <f t="shared" si="1"/>
+        <v>6.0684931506849313</v>
+      </c>
+      <c r="J13" s="2">
+        <f t="shared" si="2"/>
+        <v>1.875</v>
+      </c>
+      <c r="K13" s="2">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2">
+        <v>0</v>
+      </c>
+      <c r="M13" s="2">
+        <f t="shared" si="3"/>
+        <v>67.5</v>
+      </c>
+      <c r="N13" s="2">
+        <f t="shared" si="4"/>
+        <v>33.75</v>
+      </c>
+      <c r="O13" s="2">
+        <f t="shared" si="5"/>
+        <v>285</v>
+      </c>
+      <c r="P13" s="2">
+        <f t="shared" si="6"/>
+        <v>165</v>
+      </c>
+      <c r="Q13" s="2">
+        <f t="shared" si="7"/>
+        <v>551.25</v>
+      </c>
+      <c r="R13" s="2">
+        <f t="shared" si="8"/>
+        <v>41.34375</v>
+      </c>
+      <c r="S13" s="2">
+        <f t="shared" si="9"/>
+        <v>16.537499999999998</v>
+      </c>
+      <c r="T13" s="2">
+        <f t="shared" si="10"/>
+        <v>48.234375</v>
+      </c>
+      <c r="U13" s="2">
+        <f t="shared" si="11"/>
+        <v>39.965624999999996</v>
+      </c>
+      <c r="V13" s="2">
+        <f t="shared" si="12"/>
+        <v>979.74687499999993</v>
+      </c>
+      <c r="W13" s="2">
+        <f t="shared" si="13"/>
+        <v>146.08124999999998</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
+        <f t="shared" si="14"/>
+        <v>8</v>
+      </c>
+      <c r="B14" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="12">
+        <v>42560</v>
+      </c>
+      <c r="E14" s="10">
+        <f t="shared" si="22"/>
+        <v>46022</v>
+      </c>
+      <c r="F14" s="2">
+        <v>375</v>
+      </c>
+      <c r="G14" s="2">
+        <f t="shared" si="23"/>
+        <v>35</v>
+      </c>
+      <c r="H14" s="64">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="B13" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" s="30" t="s">
-        <v>16</v>
-      </c>
-      <c r="D13" s="12">
-        <v>43807</v>
-      </c>
-      <c r="E13" s="10">
-        <f t="shared" ref="E13:E16" si="3">+E12</f>
-        <v>46022</v>
-      </c>
-      <c r="F13" s="2">
-        <v>450</v>
-      </c>
-      <c r="G13" s="2">
-        <f t="shared" ref="G13:G16" si="4">+G11</f>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="3">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="B14" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="30" t="s">
-        <v>48</v>
-      </c>
-      <c r="D14" s="12">
-        <v>42560</v>
-      </c>
-      <c r="E14" s="10">
+      <c r="I14" s="65">
+        <f t="shared" si="1"/>
+        <v>9.4849315068493159</v>
+      </c>
+      <c r="J14" s="2">
+        <f t="shared" si="2"/>
+        <v>1.5625</v>
+      </c>
+      <c r="K14" s="2">
+        <f>+J14*2*35</f>
+        <v>109.375</v>
+      </c>
+      <c r="L14" s="2">
+        <f>+J14*2.5*20</f>
+        <v>78.125</v>
+      </c>
+      <c r="M14" s="2">
         <f t="shared" si="3"/>
-        <v>46022</v>
-      </c>
-      <c r="F14" s="2">
-        <v>375</v>
-      </c>
-      <c r="G14" s="2">
+        <v>0</v>
+      </c>
+      <c r="N14" s="2">
         <f t="shared" si="4"/>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2">
+        <f t="shared" si="5"/>
+        <v>237.5</v>
+      </c>
+      <c r="P14" s="2">
+        <f t="shared" si="6"/>
+        <v>137.5</v>
+      </c>
+      <c r="Q14" s="2">
+        <f t="shared" si="7"/>
+        <v>562.5</v>
+      </c>
+      <c r="R14" s="2">
+        <f t="shared" si="8"/>
+        <v>42.1875</v>
+      </c>
+      <c r="S14" s="2">
+        <f t="shared" si="9"/>
+        <v>16.875</v>
+      </c>
+      <c r="T14" s="2">
+        <f t="shared" si="10"/>
+        <v>49.21875</v>
+      </c>
+      <c r="U14" s="2">
+        <f t="shared" si="11"/>
+        <v>40.78125</v>
+      </c>
+      <c r="V14" s="2">
+        <f t="shared" si="12"/>
+        <v>914.84375</v>
+      </c>
+      <c r="W14" s="2">
+        <f t="shared" si="13"/>
+        <v>149.0625</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="14"/>
         <v>9</v>
       </c>
       <c r="B15" s="26" t="s">
@@ -1896,20 +2591,84 @@
         <v>42339</v>
       </c>
       <c r="E15" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="22"/>
         <v>46022</v>
       </c>
       <c r="F15" s="2">
         <v>375</v>
       </c>
       <c r="G15" s="2">
+        <f t="shared" si="23"/>
+        <v>35</v>
+      </c>
+      <c r="H15" s="64">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="I15" s="65">
+        <f t="shared" si="1"/>
+        <v>10.09041095890411</v>
+      </c>
+      <c r="J15" s="2">
+        <f t="shared" si="2"/>
+        <v>1.5625</v>
+      </c>
+      <c r="K15" s="2">
+        <f t="shared" ref="K15:K16" si="24">+J15*2*35</f>
+        <v>109.375</v>
+      </c>
+      <c r="L15" s="2">
+        <f t="shared" ref="L15:L16" si="25">+J15*2.5*20</f>
+        <v>78.125</v>
+      </c>
+      <c r="M15" s="2">
+        <f t="shared" si="3"/>
+        <v>56.25</v>
+      </c>
+      <c r="N15" s="2">
         <f t="shared" si="4"/>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+        <v>28.125</v>
+      </c>
+      <c r="O15" s="2">
+        <f t="shared" si="5"/>
+        <v>262.5</v>
+      </c>
+      <c r="P15" s="2">
+        <f t="shared" si="6"/>
+        <v>112.5</v>
+      </c>
+      <c r="Q15" s="2">
+        <f t="shared" si="7"/>
+        <v>646.875</v>
+      </c>
+      <c r="R15" s="2">
+        <f t="shared" si="8"/>
+        <v>48.515625</v>
+      </c>
+      <c r="S15" s="2">
+        <f t="shared" si="9"/>
+        <v>19.40625</v>
+      </c>
+      <c r="T15" s="2">
+        <f t="shared" si="10"/>
+        <v>56.601562499999993</v>
+      </c>
+      <c r="U15" s="2">
+        <f t="shared" si="11"/>
+        <v>46.8984375</v>
+      </c>
+      <c r="V15" s="2">
+        <f t="shared" si="12"/>
+        <v>990.5703125</v>
+      </c>
+      <c r="W15" s="2">
+        <f t="shared" si="13"/>
+        <v>171.421875</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
-        <f t="shared" si="0"/>
+        <f t="shared" si="14"/>
         <v>10</v>
       </c>
       <c r="B16" s="26" t="s">
@@ -1922,18 +2681,82 @@
         <v>41609</v>
       </c>
       <c r="E16" s="10">
-        <f t="shared" si="3"/>
+        <f t="shared" si="22"/>
         <v>46022</v>
       </c>
       <c r="F16" s="18">
         <v>395</v>
       </c>
       <c r="G16" s="2">
+        <f t="shared" si="23"/>
+        <v>35</v>
+      </c>
+      <c r="H16" s="64">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="I16" s="65">
+        <f t="shared" si="1"/>
+        <v>12.09041095890411</v>
+      </c>
+      <c r="J16" s="2">
+        <f t="shared" si="2"/>
+        <v>1.6458333333333333</v>
+      </c>
+      <c r="K16" s="2">
+        <f t="shared" si="24"/>
+        <v>115.20833333333333</v>
+      </c>
+      <c r="L16" s="2">
+        <f t="shared" si="25"/>
+        <v>82.291666666666657</v>
+      </c>
+      <c r="M16" s="2">
+        <f t="shared" si="3"/>
+        <v>59.25</v>
+      </c>
+      <c r="N16" s="2">
         <f t="shared" si="4"/>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" spans="3:7" x14ac:dyDescent="0.3">
+        <v>29.625</v>
+      </c>
+      <c r="O16" s="2">
+        <f t="shared" si="5"/>
+        <v>276.5</v>
+      </c>
+      <c r="P16" s="2">
+        <f t="shared" si="6"/>
+        <v>118.5</v>
+      </c>
+      <c r="Q16" s="2">
+        <f t="shared" si="7"/>
+        <v>681.375</v>
+      </c>
+      <c r="R16" s="2">
+        <f t="shared" si="8"/>
+        <v>51.103124999999999</v>
+      </c>
+      <c r="S16" s="2">
+        <f t="shared" si="9"/>
+        <v>20.44125</v>
+      </c>
+      <c r="T16" s="2">
+        <f t="shared" si="10"/>
+        <v>59.620312499999997</v>
+      </c>
+      <c r="U16" s="2">
+        <f t="shared" si="11"/>
+        <v>49.399687499999999</v>
+      </c>
+      <c r="V16" s="2">
+        <f t="shared" si="12"/>
+        <v>1041.5340624999999</v>
+      </c>
+      <c r="W16" s="2">
+        <f t="shared" si="13"/>
+        <v>180.56437500000001</v>
+      </c>
+    </row>
+    <row r="17" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C17" s="16"/>
       <c r="D17" s="17"/>
       <c r="E17" s="39" t="s">
@@ -1947,8 +2770,60 @@
         <f>SUM(G11:G16)</f>
         <v>210</v>
       </c>
-    </row>
-    <row r="18" spans="3:7" x14ac:dyDescent="0.3">
+      <c r="K17" s="33">
+        <f>SUM(K14:K16)</f>
+        <v>333.95833333333331</v>
+      </c>
+      <c r="L17" s="33">
+        <f>SUM(L14:L16)</f>
+        <v>238.54166666666666</v>
+      </c>
+      <c r="M17" s="33">
+        <f>SUM(M11:M16)</f>
+        <v>183</v>
+      </c>
+      <c r="N17" s="33">
+        <f t="shared" ref="N17:Q17" si="26">SUM(N11:N16)</f>
+        <v>91.5</v>
+      </c>
+      <c r="O17" s="33">
+        <f t="shared" si="26"/>
+        <v>1631.5</v>
+      </c>
+      <c r="P17" s="33">
+        <f t="shared" si="26"/>
+        <v>863.5</v>
+      </c>
+      <c r="Q17" s="33">
+        <f t="shared" si="26"/>
+        <v>3342</v>
+      </c>
+      <c r="R17" s="33">
+        <f t="shared" ref="R17" si="27">SUM(R11:R16)</f>
+        <v>250.65</v>
+      </c>
+      <c r="S17" s="33">
+        <f t="shared" ref="S17" si="28">SUM(S11:S16)</f>
+        <v>100.25999999999999</v>
+      </c>
+      <c r="T17" s="33">
+        <f t="shared" ref="T17" si="29">SUM(T11:T16)</f>
+        <v>292.42500000000001</v>
+      </c>
+      <c r="U17" s="33">
+        <f t="shared" ref="U17" si="30">SUM(U11:U16)</f>
+        <v>242.29499999999999</v>
+      </c>
+      <c r="V17" s="33">
+        <f t="shared" ref="V17" si="31">SUM(V11:V16)</f>
+        <v>5704.4449999999997</v>
+      </c>
+      <c r="W17" s="33">
+        <f t="shared" ref="W17" si="32">SUM(W11:W16)</f>
+        <v>885.63</v>
+      </c>
+    </row>
+    <row r="18" spans="3:23" x14ac:dyDescent="0.3">
       <c r="D18" s="17"/>
       <c r="E18" s="9" t="s">
         <v>11</v>
@@ -1960,6 +2835,58 @@
       <c r="G18" s="19">
         <f>G10+G17</f>
         <v>310</v>
+      </c>
+      <c r="K18" s="19">
+        <f t="shared" ref="K18:L18" si="33">+K10+K17</f>
+        <v>333.95833333333331</v>
+      </c>
+      <c r="L18" s="19">
+        <f t="shared" si="33"/>
+        <v>238.54166666666666</v>
+      </c>
+      <c r="M18" s="19">
+        <f>+M10+M17</f>
+        <v>524.25</v>
+      </c>
+      <c r="N18" s="19">
+        <f t="shared" ref="N18:Q18" si="34">+N10+N17</f>
+        <v>262.125</v>
+      </c>
+      <c r="O18" s="19">
+        <f t="shared" si="34"/>
+        <v>3970.666666666667</v>
+      </c>
+      <c r="P18" s="19">
+        <f t="shared" si="34"/>
+        <v>2049.333333333333</v>
+      </c>
+      <c r="Q18" s="19">
+        <f t="shared" si="34"/>
+        <v>7378.875</v>
+      </c>
+      <c r="R18" s="19">
+        <f t="shared" ref="R18" si="35">+R10+R17</f>
+        <v>481.41562499999998</v>
+      </c>
+      <c r="S18" s="19">
+        <f t="shared" ref="S18" si="36">+S10+S17</f>
+        <v>192.56625</v>
+      </c>
+      <c r="T18" s="19">
+        <f t="shared" ref="T18" si="37">+T10+T17</f>
+        <v>645.65156249999995</v>
+      </c>
+      <c r="U18" s="19">
+        <f t="shared" ref="U18" si="38">+U10+U17</f>
+        <v>534.96843749999994</v>
+      </c>
+      <c r="V18" s="19">
+        <f t="shared" ref="V18" si="39">+V10+V17</f>
+        <v>12981.3403125</v>
+      </c>
+      <c r="W18" s="19">
+        <f t="shared" ref="W18" si="40">+W10+W17</f>
+        <v>1854.6018749999998</v>
       </c>
     </row>
   </sheetData>
@@ -1968,6 +2895,9 @@
   <headerFooter>
     <oddFooter>&amp;L&amp;P de &amp;N</oddFooter>
   </headerFooter>
+  <ignoredErrors>
+    <ignoredError sqref="M10:P10" formula="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -2003,7 +2933,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="D1" s="56"/>
+      <c r="D1" s="55"/>
       <c r="E1" s="8" t="s">
         <v>51</v>
       </c>
@@ -2041,19 +2971,19 @@
         <v>68</v>
       </c>
       <c r="C4" s="34"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54"/>
       <c r="H4" s="35"/>
       <c r="I4" s="35"/>
-      <c r="J4" s="36"/>
-      <c r="K4" s="36"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
-      <c r="N4" s="36"/>
-      <c r="O4" s="36"/>
-      <c r="P4" s="48"/>
+      <c r="J4" s="67"/>
+      <c r="K4" s="67"/>
+      <c r="L4" s="67"/>
+      <c r="M4" s="67"/>
+      <c r="N4" s="67"/>
+      <c r="O4" s="67"/>
+      <c r="P4" s="47"/>
       <c r="Q4" s="36"/>
       <c r="R4" s="36"/>
       <c r="S4" s="36"/>
@@ -2089,28 +3019,28 @@
       <c r="I5" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="31" t="s">
+      <c r="J5" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="K5" s="31" t="s">
+      <c r="K5" s="68" t="s">
         <v>20</v>
       </c>
-      <c r="L5" s="31" t="s">
+      <c r="L5" s="68" t="s">
         <v>22</v>
       </c>
-      <c r="M5" s="31" t="s">
+      <c r="M5" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="N5" s="31" t="s">
+      <c r="N5" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="O5" s="40" t="s">
+      <c r="O5" s="71" t="s">
         <v>26</v>
       </c>
-      <c r="P5" s="49" t="s">
+      <c r="P5" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="Q5" s="45" t="s">
+      <c r="Q5" s="44" t="s">
         <v>30</v>
       </c>
       <c r="R5" s="32" t="s">
@@ -2137,7 +3067,7 @@
         <f>+EjercicioPlanilla!B6</f>
         <v>Gerencia</v>
       </c>
-      <c r="C6" s="54" t="str">
+      <c r="C6" s="53" t="str">
         <f>+EjercicioPlanilla!C6</f>
         <v>Gerente de TI</v>
       </c>
@@ -2180,11 +3110,11 @@
         <f>IF((AND($I6&gt;=1,$I6&lt;3)),((F6/30)*15),IF((AND($I6&gt;=3,$I6&lt;10)),((F6/30)*19),((F6/30)*21)))</f>
         <v>1050</v>
       </c>
-      <c r="O6" s="41">
+      <c r="O6" s="40">
         <f>IF($I6&gt;=3,($F6-N6),0)</f>
         <v>450</v>
       </c>
-      <c r="P6" s="50">
+      <c r="P6" s="49">
         <f>+F6+J6+K6+L6+M6</f>
         <v>1837.5</v>
       </c>
@@ -2222,7 +3152,7 @@
         <f>+EjercicioPlanilla!B7</f>
         <v>Administrativo</v>
       </c>
-      <c r="C7" s="54" t="str">
+      <c r="C7" s="53" t="str">
         <f>+EjercicioPlanilla!C7</f>
         <v>Asistente de gerencia</v>
       </c>
@@ -2266,11 +3196,11 @@
         <f>IF((AND($I7&gt;=1,$I7&lt;3)),((F7/30)*15),IF((AND($I7&gt;=3,$I7&lt;10)),((F7/30)*19),((F7/30)*21)))</f>
         <v>316.66666666666669</v>
       </c>
-      <c r="O7" s="41">
+      <c r="O7" s="40">
         <f t="shared" ref="O7:O9" si="1">IF($I7&gt;=3,($F7-N7),0)</f>
         <v>183.33333333333331</v>
       </c>
-      <c r="P7" s="50">
+      <c r="P7" s="49">
         <f>+F7+J7+K7+L7+M7</f>
         <v>500</v>
       </c>
@@ -2308,7 +3238,7 @@
         <f>+EjercicioPlanilla!B8</f>
         <v>Administrativo</v>
       </c>
-      <c r="C8" s="54" t="str">
+      <c r="C8" s="53" t="str">
         <f>+EjercicioPlanilla!C8</f>
         <v>Soporte de redes y HW</v>
       </c>
@@ -2352,11 +3282,11 @@
         <f>IF((AND($I8&gt;=1,$I8&lt;3)),((F8/30)*15),IF((AND($I8&gt;=3,$I8&lt;10)),((F8/30)*19),((F8/30)*21)))</f>
         <v>427.5</v>
       </c>
-      <c r="O8" s="41">
+      <c r="O8" s="40">
         <f t="shared" si="1"/>
         <v>247.5</v>
       </c>
-      <c r="P8" s="50">
+      <c r="P8" s="49">
         <f>+F8+J8+K8+L8+M8</f>
         <v>826.875</v>
       </c>
@@ -2394,7 +3324,7 @@
         <f>+EjercicioPlanilla!B9</f>
         <v>Administrativo</v>
       </c>
-      <c r="C9" s="54" t="str">
+      <c r="C9" s="53" t="str">
         <f>+EjercicioPlanilla!C9</f>
         <v>Encargado de almacenaje y seguridad de la información</v>
       </c>
@@ -2438,11 +3368,11 @@
         <f>IF((AND($I9&gt;=1,$I9&lt;3)),((F9/30)*15),IF((AND($I9&gt;=3,$I9&lt;10)),((F9/30)*19),((F9/30)*21)))</f>
         <v>475</v>
       </c>
-      <c r="O9" s="41">
+      <c r="O9" s="40">
         <f t="shared" si="1"/>
         <v>275</v>
       </c>
-      <c r="P9" s="50">
+      <c r="P9" s="49">
         <f>+F9+J9+K9+L9+M9</f>
         <v>750</v>
       </c>
@@ -2515,15 +3445,15 @@
         <f t="shared" ref="N10:V10" si="6">SUM(N6:N9)</f>
         <v>2269.166666666667</v>
       </c>
-      <c r="O10" s="42">
+      <c r="O10" s="41">
         <f t="shared" si="6"/>
         <v>1155.8333333333333</v>
       </c>
-      <c r="P10" s="51">
+      <c r="P10" s="50">
         <f>SUM(P6:P9)</f>
         <v>3914.375</v>
       </c>
-      <c r="Q10" s="46">
+      <c r="Q10" s="45">
         <f>SUM(Q6:Q9)</f>
         <v>230.765625</v>
       </c>
@@ -2557,7 +3487,7 @@
         <f>+EjercicioPlanilla!B11</f>
         <v>Operaciones</v>
       </c>
-      <c r="C11" s="54" t="str">
+      <c r="C11" s="53" t="str">
         <f>+EjercicioPlanilla!C11</f>
         <v>Supervisor de occidente</v>
       </c>
@@ -2601,11 +3531,11 @@
         <f t="shared" ref="N11:N16" si="11">IF((AND($I11&gt;=1,$I11&lt;3)),((F11/30)*15),IF((AND($I11&gt;=3,$I11&lt;10)),((F11/30)*19),((F11/30)*21)))</f>
         <v>300.83333333333337</v>
       </c>
-      <c r="O11" s="41">
+      <c r="O11" s="40">
         <f t="shared" ref="O11:O16" si="12">IF($I11&gt;=3,($F11-N11),0)</f>
         <v>174.16666666666663</v>
       </c>
-      <c r="P11" s="50">
+      <c r="P11" s="49">
         <f t="shared" ref="P11:P16" si="13">+F11+J11+K11+L11+M11</f>
         <v>475</v>
       </c>
@@ -2643,7 +3573,7 @@
         <f>+EjercicioPlanilla!B12</f>
         <v>Operaciones</v>
       </c>
-      <c r="C12" s="54" t="str">
+      <c r="C12" s="53" t="str">
         <f>+EjercicioPlanilla!C12</f>
         <v>Supervisor de oriente</v>
       </c>
@@ -2687,11 +3617,11 @@
         <f t="shared" si="11"/>
         <v>269.16666666666663</v>
       </c>
-      <c r="O12" s="41">
+      <c r="O12" s="40">
         <f t="shared" si="12"/>
         <v>155.83333333333337</v>
       </c>
-      <c r="P12" s="50">
+      <c r="P12" s="49">
         <f t="shared" si="13"/>
         <v>425</v>
       </c>
@@ -2729,7 +3659,7 @@
         <f>+EjercicioPlanilla!B13</f>
         <v>Operaciones</v>
       </c>
-      <c r="C13" s="54" t="str">
+      <c r="C13" s="53" t="str">
         <f>+EjercicioPlanilla!C13</f>
         <v>Supervisor centro</v>
       </c>
@@ -2773,11 +3703,11 @@
         <f t="shared" si="11"/>
         <v>285</v>
       </c>
-      <c r="O13" s="41">
+      <c r="O13" s="40">
         <f t="shared" si="12"/>
         <v>165</v>
       </c>
-      <c r="P13" s="50">
+      <c r="P13" s="49">
         <f t="shared" si="13"/>
         <v>551.25</v>
       </c>
@@ -2815,7 +3745,7 @@
         <f>+EjercicioPlanilla!B14</f>
         <v>Operaciones</v>
       </c>
-      <c r="C14" s="54" t="str">
+      <c r="C14" s="53" t="str">
         <f>+EjercicioPlanilla!C14</f>
         <v>Técnico de soporte a domicilio-Occidente</v>
       </c>
@@ -2862,11 +3792,11 @@
         <f t="shared" si="11"/>
         <v>285</v>
       </c>
-      <c r="O14" s="41">
+      <c r="O14" s="40">
         <f t="shared" si="12"/>
         <v>165</v>
       </c>
-      <c r="P14" s="50">
+      <c r="P14" s="49">
         <f t="shared" si="13"/>
         <v>675</v>
       </c>
@@ -2904,7 +3834,7 @@
         <f>+EjercicioPlanilla!B15</f>
         <v>Operaciones</v>
       </c>
-      <c r="C15" s="54" t="str">
+      <c r="C15" s="53" t="str">
         <f>+EjercicioPlanilla!C15</f>
         <v>Técnico de soporte a domicilio-Oriente</v>
       </c>
@@ -2951,11 +3881,11 @@
         <f t="shared" si="11"/>
         <v>350</v>
       </c>
-      <c r="O15" s="41">
+      <c r="O15" s="40">
         <f t="shared" si="12"/>
         <v>150</v>
       </c>
-      <c r="P15" s="50">
+      <c r="P15" s="49">
         <f t="shared" si="13"/>
         <v>862.5</v>
       </c>
@@ -2993,7 +3923,7 @@
         <f>+EjercicioPlanilla!B16</f>
         <v>Operaciones</v>
       </c>
-      <c r="C16" s="54" t="str">
+      <c r="C16" s="53" t="str">
         <f>+EjercicioPlanilla!C16</f>
         <v>Técnico de soportea domicilio-Central</v>
       </c>
@@ -3040,11 +3970,11 @@
         <f t="shared" si="11"/>
         <v>315</v>
       </c>
-      <c r="O16" s="41">
+      <c r="O16" s="40">
         <f t="shared" si="12"/>
         <v>135</v>
       </c>
-      <c r="P16" s="50">
+      <c r="P16" s="49">
         <f t="shared" si="13"/>
         <v>776.25</v>
       </c>
@@ -3109,15 +4039,15 @@
         <f t="shared" si="22"/>
         <v>1805</v>
       </c>
-      <c r="O17" s="43">
+      <c r="O17" s="42">
         <f t="shared" ref="O17:P17" si="24">SUM(O11:O16)</f>
         <v>945</v>
       </c>
-      <c r="P17" s="52">
+      <c r="P17" s="51">
         <f t="shared" si="24"/>
         <v>3765</v>
       </c>
-      <c r="Q17" s="47">
+      <c r="Q17" s="46">
         <f>SUM(Q11:Q16)</f>
         <v>282.375</v>
       </c>
@@ -3177,11 +4107,11 @@
         <f t="shared" si="26"/>
         <v>4074.166666666667</v>
       </c>
-      <c r="O18" s="44">
+      <c r="O18" s="43">
         <f t="shared" ref="O18:P18" si="28">+O10+O17</f>
         <v>2100.833333333333</v>
       </c>
-      <c r="P18" s="53">
+      <c r="P18" s="52">
         <f t="shared" si="28"/>
         <v>7679.375</v>
       </c>

</xml_diff>